<commit_message>
Fix: Remove pandas dependency, use pure openpyxl in batch_data_processor.py
</commit_message>
<xml_diff>
--- a/auto_input_queue.xlsx
+++ b/auto_input_queue.xlsx
@@ -27,13 +27,13 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -76,13 +76,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,22 +511,22 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>3405010201</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>900002933363</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -531,12 +534,12 @@
       <c r="F2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002933363] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [100] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -546,22 +549,22 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>3405010201</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>900002933362</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -569,12 +572,12 @@
       <c r="F3" s="2" t="n">
         <v>175</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002933362] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [175] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -584,22 +587,22 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>3405030101</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>900002995780</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -607,12 +610,12 @@
       <c r="F4" s="2" t="n">
         <v>361</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002995780] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [361] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -622,22 +625,22 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>3405040101</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>999900002402</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -645,12 +648,12 @@
       <c r="F5" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002402] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [330] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -660,22 +663,22 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>3405100201</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>900002908260</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -683,12 +686,12 @@
       <c r="F6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002908260] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [30] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -698,22 +701,22 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>3405100201</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>999900003477</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -721,12 +724,12 @@
       <c r="F7" s="2" t="n">
         <v>110</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900003477] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [110] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -736,22 +739,22 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3405100201</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>999900002518</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -759,12 +762,12 @@
       <c r="F8" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002518] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [420] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -774,22 +777,22 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3405110101</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>100006174226</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -797,12 +800,12 @@
       <c r="F9" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006174226] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -812,22 +815,22 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>3405120101</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>199900015444</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -835,12 +838,12 @@
       <c r="F10" s="2" t="n">
         <v>280</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Gõ [199900015444] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [280] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -850,22 +853,22 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>3405130101</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>999900003269</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -873,12 +876,12 @@
       <c r="F11" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900003269] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -888,22 +891,22 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>3405210301</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>100006145580</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -911,12 +914,12 @@
       <c r="F12" s="2" t="n">
         <v>1240</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006145580] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [1240] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -926,22 +929,22 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>3405230101</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>100006145575</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -949,12 +952,12 @@
       <c r="F13" s="2" t="n">
         <v>615</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006145575] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [615] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -964,22 +967,22 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>3405350001</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>999900004488</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -987,12 +990,12 @@
       <c r="F14" s="2" t="n">
         <v>497</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900004488] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [497] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1002,22 +1005,22 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>3405360001</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>999900002815</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1025,12 +1028,12 @@
       <c r="F15" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002815] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [75] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1040,22 +1043,22 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>3405360001</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>100006024592</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1063,12 +1066,12 @@
       <c r="F16" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006024592] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [120] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1078,22 +1081,22 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>3407810101</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>199900015677</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1101,12 +1104,12 @@
       <c r="F17" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Gõ [199900015677] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [70] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1116,22 +1119,22 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>3407810101</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>100005985324</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1139,12 +1142,12 @@
       <c r="F18" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Gõ [100005985324] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [200] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1154,22 +1157,22 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>3407810101</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>199900015061</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1177,12 +1180,12 @@
       <c r="F19" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Gõ [199900015061] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [400] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1192,22 +1195,22 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>3407820101</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>199900015062</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1215,12 +1218,12 @@
       <c r="F20" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Gõ [199900015062] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [250] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1230,22 +1233,22 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>3407830101</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>100006014820</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1253,12 +1256,12 @@
       <c r="F21" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006014820] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1268,22 +1271,22 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>3407840101</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>100006005711</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1291,12 +1294,12 @@
       <c r="F22" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006005711] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1306,22 +1309,22 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>3407880001</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>999900001668</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1329,12 +1332,12 @@
       <c r="F23" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900001668] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [200] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1344,22 +1347,22 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>3423020001</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>999900004498</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1367,12 +1370,12 @@
       <c r="F24" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900004498] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [34] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1382,22 +1385,22 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>3423130001</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>999900004385</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1405,12 +1408,12 @@
       <c r="F25" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900004385] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [400] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1420,22 +1423,22 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>3423140001</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>900002994643</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1443,12 +1446,12 @@
       <c r="F26" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002994643] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [230] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1458,22 +1461,22 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>3447230001</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>900002965733</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1481,12 +1484,12 @@
       <c r="F27" s="2" t="n">
         <v>1310</v>
       </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002965733] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [1310] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1496,22 +1499,22 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>3447270001</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>999900002763</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1519,12 +1522,12 @@
       <c r="F28" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002763] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [100] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1534,22 +1537,22 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>3447270001</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>999900001722</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1557,12 +1560,12 @@
       <c r="F29" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900001722] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1572,22 +1575,22 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>3447270001</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>900002900191</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1595,12 +1598,12 @@
       <c r="F30" s="2" t="n">
         <v>1203</v>
       </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002900191] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [1203] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1610,22 +1613,22 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>3447510001</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>900002999886</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1633,12 +1636,12 @@
       <c r="F31" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002999886] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [46] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1648,22 +1651,22 @@
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>3447520001</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>900002985139</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1671,12 +1674,12 @@
       <c r="F32" s="2" t="n">
         <v>964</v>
       </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002985139] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [964] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1686,22 +1689,22 @@
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>3447530001</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>999900004514</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1709,12 +1712,12 @@
       <c r="F33" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900004514] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [420] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1724,22 +1727,22 @@
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>3447530001</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>900003000594</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1747,12 +1750,12 @@
       <c r="F34" s="2" t="n">
         <v>490</v>
       </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Gõ [900003000594] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [490] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1762,22 +1765,22 @@
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>3447530001</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>999900002544</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1785,12 +1788,12 @@
       <c r="F35" s="2" t="n">
         <v>560</v>
       </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002544] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [560] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1800,22 +1803,22 @@
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>3447970001</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>999900003410</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1823,12 +1826,12 @@
       <c r="F36" s="2" t="n">
         <v>890</v>
       </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900003410] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [890] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1838,22 +1841,22 @@
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>3447990001</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>999900002901</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1861,12 +1864,12 @@
       <c r="F37" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002901] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [70] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1876,22 +1879,22 @@
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>3447990001</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>100006183153</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1899,12 +1902,12 @@
       <c r="F38" s="2" t="n">
         <v>210</v>
       </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006183153] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [210] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1914,22 +1917,22 @@
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>3447990001</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>100005975074</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1937,12 +1940,12 @@
       <c r="F39" s="2" t="n">
         <v>570</v>
       </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Gõ [100005975074] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [570] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1952,22 +1955,22 @@
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>3448000001</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>100006183151</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -1975,12 +1978,12 @@
       <c r="F40" s="2" t="n">
         <v>210</v>
       </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006183151] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [210] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -1990,22 +1993,22 @@
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>3448000001</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>100006165237</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2013,12 +2016,12 @@
       <c r="F41" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006165237] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [300] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2028,22 +2031,22 @@
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>3448000001</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>100005975075</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2051,12 +2054,12 @@
       <c r="F42" s="2" t="n">
         <v>570</v>
       </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>Gõ [100005975075] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [570] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2066,22 +2069,22 @@
       <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>3451270001</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>999900001686</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2089,12 +2092,12 @@
       <c r="F43" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900001686] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2104,22 +2107,22 @@
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>3451280001</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>999900003221</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2127,12 +2130,12 @@
       <c r="F44" s="2" t="n">
         <v>290</v>
       </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900003221] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [290] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2142,22 +2145,22 @@
       <c r="A45" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>3453530001</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>900002996654</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2165,12 +2168,12 @@
       <c r="F45" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002996654] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [600] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2180,22 +2183,22 @@
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>3453530001</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>900002897510</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2203,12 +2206,12 @@
       <c r="F46" s="2" t="n">
         <v>855</v>
       </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002897510] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [855] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2218,22 +2221,22 @@
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>3464230001</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>999900002997</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2241,12 +2244,12 @@
       <c r="F47" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002997] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [20] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2256,22 +2259,22 @@
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>3464670001</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>900002989157</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2279,12 +2282,12 @@
       <c r="F48" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002989157] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2294,22 +2297,22 @@
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>3464670001</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>900002998555</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2317,12 +2320,12 @@
       <c r="F49" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002998555] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [1000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2332,22 +2335,22 @@
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>3464730001</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>999900003520</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2355,12 +2358,12 @@
       <c r="F50" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900003520] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [100] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2370,22 +2373,22 @@
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>3465830001</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>999900002864</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2393,12 +2396,12 @@
       <c r="F51" s="2" t="n">
         <v>650</v>
       </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002864] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [650] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2408,22 +2411,22 @@
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>3465960101</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>900002997933</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2431,12 +2434,12 @@
       <c r="F52" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002997933] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [59] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2446,22 +2449,22 @@
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>3465960101</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>900002997930</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2469,12 +2472,12 @@
       <c r="F53" s="2" t="n">
         <v>352</v>
       </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002997930] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [352] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2484,22 +2487,22 @@
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>3465990001</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>999900002982</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2507,12 +2510,12 @@
       <c r="F54" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002982] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [400] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2522,22 +2525,22 @@
       <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>5100630051</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>999900002368</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2545,12 +2548,12 @@
       <c r="F55" s="2" t="n">
         <v>669</v>
       </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002368] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [669] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2560,22 +2563,22 @@
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>7100060051</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>900002991674</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2583,12 +2586,12 @@
       <c r="F56" s="2" t="n">
         <v>1489</v>
       </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002991674] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [1489] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2598,22 +2601,22 @@
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>7100060051PA</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>100006083597</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2621,12 +2624,12 @@
       <c r="F57" s="2" t="n">
         <v>24500</v>
       </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006083597] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [24500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2636,22 +2639,22 @@
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>7101130051</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>900003001800</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2659,12 +2662,12 @@
       <c r="F58" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>Gõ [900003001800] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [2000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2674,22 +2677,22 @@
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>7109830051PD</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>100006167735</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2697,12 +2700,12 @@
       <c r="F59" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>Gõ [100006167735] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [2000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2712,22 +2715,22 @@
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>7150110001</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>999900002062</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2735,12 +2738,12 @@
       <c r="F60" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002062] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [3000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2750,22 +2753,22 @@
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>7150110001</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>900002918838</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2773,12 +2776,12 @@
       <c r="F61" s="2" t="n">
         <v>4000</v>
       </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002918838] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [4000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2788,22 +2791,22 @@
       <c r="A62" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>7150150001</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>999900002111</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2811,12 +2814,12 @@
       <c r="F62" s="2" t="n">
         <v>1900</v>
       </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002111] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [1900] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2826,22 +2829,22 @@
       <c r="A63" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>7150180001</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>999900002208</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2849,12 +2852,12 @@
       <c r="F63" s="2" t="n">
         <v>7700</v>
       </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002208] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [7700] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2864,22 +2867,22 @@
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>7150200001</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>999900002608</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -2887,12 +2890,12 @@
       <c r="F64" s="2" t="n">
         <v>8000</v>
       </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002608] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [8000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2902,22 +2905,22 @@
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>7150780201</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>900002908864</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -2925,12 +2928,12 @@
       <c r="F65" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002908864] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [200] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2940,22 +2943,22 @@
       <c r="A66" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>7151480001</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>900002917491</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -2963,12 +2966,12 @@
       <c r="F66" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002917491] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [200] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -2978,22 +2981,22 @@
       <c r="A67" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>7151480001</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>999900002262</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -3001,12 +3004,12 @@
       <c r="F67" s="2" t="n">
         <v>550</v>
       </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002262] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [550] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -3016,22 +3019,22 @@
       <c r="A68" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>7156770001</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>999900002139</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -3039,12 +3042,12 @@
       <c r="F68" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002139] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [12000] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -3054,22 +3057,22 @@
       <c r="A69" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>7156770001</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>999900002103</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -3077,12 +3080,12 @@
       <c r="F69" s="2" t="n">
         <v>18500</v>
       </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002103] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [18500] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -3092,22 +3095,22 @@
       <c r="A70" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>7200260001</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>999900005354</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -3115,12 +3118,12 @@
       <c r="F70" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900005354] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [1] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -3130,22 +3133,22 @@
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>7200260001</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>999900002280</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -3153,12 +3156,12 @@
       <c r="F71" s="2" t="n">
         <v>499</v>
       </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>Gõ [999900002280] -&gt; Enter -&gt; Gõ [50] -&gt; Enter -&gt; Gõ [499] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>
@@ -3168,22 +3171,22 @@
       <c r="A72" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>7200260001</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>900002997924</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -3191,12 +3194,12 @@
       <c r="F72" s="2" t="n">
         <v>989</v>
       </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
         <is>
           <t>Gõ [900002997924] -&gt; Enter -&gt; Gõ [62] -&gt; Enter -&gt; Gõ [989] -&gt; Enter -&gt; Gõ [01] -&gt; Enter x 4</t>
         </is>

</xml_diff>